<commit_message>
chore(results): refresh the profiling workbook after the fix
</commit_message>
<xml_diff>
--- a/results/01_profiling.xlsx
+++ b/results/01_profiling.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="46">
   <si>
     <t>Partition</t>
   </si>
@@ -39,85 +39,121 @@
     <t>Holdout</t>
   </si>
   <si>
+    <t>Predictor</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Median / n(=1)</t>
+  </si>
+  <si>
+    <t>IQR / % of records</t>
+  </si>
+  <si>
+    <t>Range</t>
+  </si>
+  <si>
+    <t>Skew</t>
+  </si>
+  <si>
+    <t>Outliers(1.5IQR)</t>
+  </si>
+  <si>
+    <t>Missing</t>
+  </si>
+  <si>
+    <t>AGE</t>
+  </si>
+  <si>
+    <t>ANNUALCONTRIBUTION</t>
+  </si>
+  <si>
+    <t>ANNUALCLAIMAMOUNT</t>
+  </si>
+  <si>
+    <t>UNITSTOTAL</t>
+  </si>
+  <si>
+    <t>GENDER_M</t>
+  </si>
+  <si>
+    <t>SCHEMETYPE_MEDIUM</t>
+  </si>
+  <si>
+    <t>SCHEMETYPE_PREMIUM</t>
+  </si>
+  <si>
+    <t>DIAGNOSIS_HYPERTENSION</t>
+  </si>
+  <si>
+    <t>COVERTYPE_STANDARD</t>
+  </si>
+  <si>
+    <t>COMORBIDITY_NO_COMORBIDITY</t>
+  </si>
+  <si>
+    <t>COMPLICATIONDEVELOPMENT_NO_COMPLICATION</t>
+  </si>
+  <si>
+    <t>Cont.</t>
+  </si>
+  <si>
+    <t>Bin.</t>
+  </si>
+  <si>
+    <t>[46.0, 66.0]</t>
+  </si>
+  <si>
+    <t>[2,718,696.0, 6,889,900.0]</t>
+  </si>
+  <si>
+    <t>[12,337.3, 102,120.1]</t>
+  </si>
+  <si>
+    <t>[120.0, 720.0]</t>
+  </si>
+  <si>
+    <t>54.3%</t>
+  </si>
+  <si>
+    <t>21.4%</t>
+  </si>
+  <si>
+    <t>74.3%</t>
+  </si>
+  <si>
+    <t>80.0%</t>
+  </si>
+  <si>
+    <t>71.0%</t>
+  </si>
+  <si>
+    <t>90.4%</t>
+  </si>
+  <si>
+    <t>16.0-103.0</t>
+  </si>
+  <si>
+    <t>211,764.0-11,770,788.0</t>
+  </si>
+  <si>
+    <t>1.0-9,401,312,187.4</t>
+  </si>
+  <si>
+    <t>1.0-21,290,640.0</t>
+  </si>
+  <si>
+    <t>0-1</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
     <t>Feature</t>
   </si>
   <si>
-    <t>Median</t>
-  </si>
-  <si>
-    <t>IQR</t>
-  </si>
-  <si>
-    <t>Range</t>
-  </si>
-  <si>
-    <t>Skew</t>
-  </si>
-  <si>
-    <t>Outliers(1.5IQR)</t>
-  </si>
-  <si>
-    <t>Missing</t>
-  </si>
-  <si>
-    <t>AGE</t>
-  </si>
-  <si>
-    <t>ANNUALCONTRIBUTION</t>
-  </si>
-  <si>
-    <t>ANNUALCLAIMAMOUNT</t>
-  </si>
-  <si>
-    <t>UNITSTOTAL</t>
-  </si>
-  <si>
-    <t>[46, 66]</t>
-  </si>
-  <si>
-    <t>[2718696, 6889900]</t>
-  </si>
-  <si>
-    <t>[12299, 102120]</t>
-  </si>
-  <si>
-    <t>[120, 720]</t>
-  </si>
-  <si>
-    <t>16-103</t>
-  </si>
-  <si>
-    <t>211764-11770788</t>
-  </si>
-  <si>
-    <t>1-1299691096</t>
-  </si>
-  <si>
-    <t>1-12847800</t>
-  </si>
-  <si>
     <t>Corr_with_target</t>
-  </si>
-  <si>
-    <t>COMORBIDITY_NO_COMORBIDITY</t>
-  </si>
-  <si>
-    <t>SCHEMETYPE_MEDIUM</t>
-  </si>
-  <si>
-    <t>COMPLICATIONDEVELOPMENT_NO_COMPLICATION</t>
-  </si>
-  <si>
-    <t>DIAGNOSIS_HYPERTENSION</t>
-  </si>
-  <si>
-    <t>GENDER_M</t>
-  </si>
-  <si>
-    <t>COVERTYPE_STANDARD</t>
-  </si>
-  <si>
-    <t>SCHEMETYPE_PREMIUM</t>
   </si>
 </sst>
 </file>
@@ -541,10 +577,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -566,96 +602,293 @@
       <c r="G1" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2">
+        <v>15</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2">
         <v>56</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2">
+        <v>0.16</v>
+      </c>
+      <c r="G2">
+        <v>13</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3">
+        <v>6889900</v>
+      </c>
+      <c r="D3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3">
+        <v>-0.67</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4">
+        <v>40482</v>
+      </c>
+      <c r="D4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4">
+        <v>150.35</v>
+      </c>
+      <c r="G4">
+        <v>2447</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
         <v>18</v>
       </c>
-      <c r="D2" t="s">
+      <c r="B5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5">
+        <v>345</v>
+      </c>
+      <c r="D5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F5">
+        <v>102.79</v>
+      </c>
+      <c r="G5">
+        <v>1556</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6">
+        <v>13063</v>
+      </c>
+      <c r="D6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F6" t="s">
+        <v>43</v>
+      </c>
+      <c r="G6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7">
+        <v>5146</v>
+      </c>
+      <c r="D7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" t="s">
+        <v>42</v>
+      </c>
+      <c r="F7" t="s">
+        <v>43</v>
+      </c>
+      <c r="G7" t="s">
+        <v>43</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8">
+        <v>17882</v>
+      </c>
+      <c r="D8" t="s">
+        <v>34</v>
+      </c>
+      <c r="E8" t="s">
+        <v>42</v>
+      </c>
+      <c r="F8" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" t="s">
+        <v>43</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" t="s">
         <v>22</v>
       </c>
-      <c r="E2">
-        <v>0.2</v>
-      </c>
-      <c r="F2">
-        <v>12</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3">
-        <v>6889900</v>
-      </c>
-      <c r="C3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9">
+        <v>19266</v>
+      </c>
+      <c r="D9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E9" t="s">
+        <v>42</v>
+      </c>
+      <c r="F9" t="s">
+        <v>43</v>
+      </c>
+      <c r="G9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" t="s">
         <v>23</v>
       </c>
-      <c r="E3">
-        <v>-0.7</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4">
-        <v>40291.1</v>
-      </c>
-      <c r="C4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="B10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10">
+        <v>19261</v>
+      </c>
+      <c r="D10" t="s">
+        <v>35</v>
+      </c>
+      <c r="E10" t="s">
+        <v>42</v>
+      </c>
+      <c r="F10" t="s">
+        <v>43</v>
+      </c>
+      <c r="G10" t="s">
+        <v>43</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" t="s">
         <v>24</v>
       </c>
-      <c r="E4">
-        <v>111.2</v>
-      </c>
-      <c r="F4">
-        <v>1959</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5">
-        <v>336</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11">
+        <v>17096</v>
+      </c>
+      <c r="D11" t="s">
+        <v>36</v>
+      </c>
+      <c r="E11" t="s">
+        <v>42</v>
+      </c>
+      <c r="F11" t="s">
+        <v>43</v>
+      </c>
+      <c r="G11" t="s">
+        <v>43</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" t="s">
         <v>25</v>
       </c>
-      <c r="E5">
-        <v>99.2</v>
-      </c>
-      <c r="F5">
-        <v>1243</v>
-      </c>
-      <c r="G5">
+      <c r="B12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12">
+        <v>21760</v>
+      </c>
+      <c r="D12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" t="s">
+        <v>42</v>
+      </c>
+      <c r="F12" t="s">
+        <v>43</v>
+      </c>
+      <c r="G12" t="s">
+        <v>43</v>
+      </c>
+      <c r="H12">
         <v>0</v>
       </c>
     </row>
@@ -671,15 +904,15 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B2">
         <v>-0.1401143588239721</v>
@@ -687,7 +920,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B3">
         <v>-0.03970732418770358</v>
@@ -695,7 +928,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B4">
         <v>-0.03662367026541147</v>
@@ -703,7 +936,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B5">
         <v>-0.03594024733414995</v>
@@ -711,7 +944,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="B6">
         <v>-0.03003731290529533</v>
@@ -719,7 +952,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B7">
         <v>-0.002485438844006576</v>
@@ -727,7 +960,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B8">
         <v>0.00510309689929852</v>
@@ -735,7 +968,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="B9">
         <v>0.008247597370403537</v>
@@ -743,7 +976,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B10">
         <v>0.04367889660912529</v>
@@ -751,7 +984,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B11">
         <v>0.05312218532024194</v>
@@ -759,7 +992,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B12">
         <v>0.237222063181109</v>

</xml_diff>